<commit_message>
ingest: resolve Grandeur ambiguous row to live SPC-GRAN-0001
Albert confirmed the price list's "8936" is the same product as the live
"GF8936". Adopted the live record in both files: SKU SPC-GRAN-0001,
handle GRND7ATLANTICGF8936, Lightspeed ID, Supplier SKU GF8936 and
product name, per RULE 0/0a. New price data from the list is retained;
the ambiguity warning in Salesperson notes is replaced with a
resolution note.

Final state of both files:
  213 matched — every LS id and handle verified identical to live
   18 new     — LS id blank (correct; LS assigns on import), minted handles
    0 ambiguous, 0 placeholder GRND-prefixed SKUs remaining
  SKUs and handles unique, all handles alphanumeric
  LS file id/handle/sku consistent with the Airtable file on every row

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DXeoXeeCbDbxXN7V7sibfF
</commit_message>
<xml_diff>
--- a/ingest/2026-09-03/grandeur_airtable_upload_2026-09-03.xlsx
+++ b/ingest/2026-09-03/grandeur_airtable_upload_2026-09-03.xlsx
@@ -13581,12 +13581,12 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>GRNDLVP-0002</t>
+          <t>SPC-GRAN-0001</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Grandeur 7" Atlantic — 8936</t>
+          <t>Grandeur 7" Atlantic — GF8936</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -13601,12 +13601,17 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>8936</t>
+          <t>GF8936</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>3f1ed949-8615-4feb-b12c-ec27fcec7287</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>GRND7ATLANTIC8936</t>
+          <t>GRND7ATLANTICGF8936</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -13706,12 +13711,17 @@
       </c>
       <c r="BC104" t="inlineStr">
         <is>
-          <t>AMBIGUOUS MATCH — could not be reconciled against the live catalogue with confidence; SKU below is the run-generated placeholder, NOT a real catalogue SKU. Colour placeholder "8936" vs live "GF8936" (SPC-GRAN-0001, Supplier SKU GF8936). Partial supplier-code match only — not confident enough to adopt. Confirm with Grandeur, then either adopt SPC-GRAN-0001 or keep as new. Resolve before import. | Colour name not provided by supplier -- product identified only by code '8936'. Used as colour placeholder; confirm actual colour name with Grandeur. SALE item, no regular equivalent in this collection -&gt; Cost/unit=SALE price per Sale rule 3. Composition: 4.0mm SPC + 1mm underpad (material not named). *Two-side Closed Treads Available.</t>
+          <t>Resolved 2026-09-03 (Albert): adopted live SPC-GRAN-0001 — price-list code "8936" confirmed as the same product as live "GF8936". SKU, LS handle, Lightspeed ID and Supplier SKU taken from the live record per RULE 0. Colour name not provided by supplier -- product identified only by code '8936'. Used as colour placeholder; confirm actual colour name with Grandeur. SALE item, no regular equivalent in this collection -&gt; Cost/unit=SALE price per Sale rule 3. Composition: 4.0mm SPC + 1mm underpad (material not named). *Two-side Closed Treads Available.</t>
+        </is>
+      </c>
+      <c r="BE104" t="inlineStr">
+        <is>
+          <t>rec71K5yB4qVmqrnm</t>
         </is>
       </c>
       <c r="BF104" t="inlineStr">
         <is>
-          <t>ambiguous</t>
+          <t>matched</t>
         </is>
       </c>
     </row>

</xml_diff>